<commit_message>
Add test tooling, update packages, and normalize logs
Add and configure testing tooling, update frontend dependencies, and expand clock log normalization. Relax ESLint rules for test files and switch jest.setup to CommonJS require; add a jest.d.ts declaration. Update package.json/package-lock to include Jest and Testing Library packages and many updated transitive deps. Add a valid attendance sample XLSX and adjust frontend tests/pages/hooks accordingly. Extend backend clockLogNormalization IN/OUT type sets with additional Spanish/variant lunch synonyms to improve log categorization.
</commit_message>
<xml_diff>
--- a/src/frontend/public/samples/attendance-sample-3emp-15days.xlsx
+++ b/src/frontend/public/samples/attendance-sample-3emp-15days.xlsx
@@ -1,10 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92B76821-932A-45BD-9F3B-560056C6B206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="28680" yWindow="-1155" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Marcas Asistencia" state="visible" r:id="rId4"/>
+    <sheet name="Marcas Asistencia" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -25,15 +29,9 @@
     <t>2026-04-01 08:00:00</t>
   </si>
   <si>
-    <t>ENTRADA</t>
-  </si>
-  <si>
     <t>2026-04-01 12:00:00</t>
   </si>
   <si>
-    <t>SALIDA</t>
-  </si>
-  <si>
     <t>2026-04-01 13:00:00</t>
   </si>
   <si>
@@ -239,23 +237,31 @@
   </si>
   <si>
     <t>2026-04-04 17:00:00</t>
+  </si>
+  <si>
+    <t>IN</t>
+  </si>
+  <si>
+    <t>OUT</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="3">
@@ -293,7 +299,9 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{AC792F5B-9A4E-4396-AD67-0BA00C518950}"/>
+  </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -626,9 +634,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C110"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="20" style="1" customWidth="1"/>
@@ -654,7 +662,7 @@
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -662,10 +670,10 @@
         <v>101</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -673,10 +681,10 @@
         <v>101</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -684,10 +692,10 @@
         <v>101</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -695,10 +703,10 @@
         <v>101</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C6" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -706,10 +714,10 @@
         <v>101</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -717,10 +725,10 @@
         <v>101</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C8" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -728,10 +736,10 @@
         <v>101</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C9" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -739,10 +747,10 @@
         <v>101</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C10" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -750,10 +758,10 @@
         <v>101</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C11" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -761,10 +769,10 @@
         <v>101</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C12" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -772,10 +780,10 @@
         <v>101</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C13" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -783,10 +791,10 @@
         <v>101</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C14" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -794,10 +802,10 @@
         <v>101</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C15" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -805,10 +813,10 @@
         <v>101</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C16" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -816,10 +824,10 @@
         <v>101</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C17" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -827,10 +835,10 @@
         <v>101</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C18" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -838,10 +846,10 @@
         <v>101</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C19" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -849,10 +857,10 @@
         <v>101</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C20" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -860,10 +868,10 @@
         <v>101</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C21" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -871,10 +879,10 @@
         <v>101</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C22" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -882,10 +890,10 @@
         <v>101</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C23" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -893,10 +901,10 @@
         <v>101</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C24" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -904,10 +912,10 @@
         <v>101</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C25" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -915,10 +923,10 @@
         <v>101</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C26" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -926,10 +934,10 @@
         <v>101</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C27" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -937,10 +945,10 @@
         <v>101</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C28" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -948,10 +956,10 @@
         <v>101</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C29" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -959,10 +967,10 @@
         <v>101</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C30" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -970,10 +978,10 @@
         <v>101</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C31" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -981,10 +989,10 @@
         <v>101</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C32" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -992,10 +1000,10 @@
         <v>101</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C33" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -1003,10 +1011,10 @@
         <v>101</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C34" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -1014,10 +1022,10 @@
         <v>101</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C35" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -1025,10 +1033,10 @@
         <v>101</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C36" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -1036,10 +1044,10 @@
         <v>101</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C37" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -1047,10 +1055,10 @@
         <v>101</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C38" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -1058,10 +1066,10 @@
         <v>101</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C39" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -1069,10 +1077,10 @@
         <v>101</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C40" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -1080,10 +1088,10 @@
         <v>101</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C41" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -1091,10 +1099,10 @@
         <v>101</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C42" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -1102,10 +1110,10 @@
         <v>101</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C43" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -1113,10 +1121,10 @@
         <v>101</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C44" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -1124,10 +1132,10 @@
         <v>101</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C45" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
@@ -1135,10 +1143,10 @@
         <v>102</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C46" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -1146,10 +1154,10 @@
         <v>102</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C47" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -1157,10 +1165,10 @@
         <v>102</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C48" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -1168,10 +1176,10 @@
         <v>102</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C49" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -1179,10 +1187,10 @@
         <v>102</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C50" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -1190,10 +1198,10 @@
         <v>102</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C51" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
@@ -1201,10 +1209,10 @@
         <v>102</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C52" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
@@ -1212,10 +1220,10 @@
         <v>102</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C53" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
@@ -1223,10 +1231,10 @@
         <v>102</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C54" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
@@ -1234,10 +1242,10 @@
         <v>102</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C55" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
@@ -1245,10 +1253,10 @@
         <v>102</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C56" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
@@ -1256,10 +1264,10 @@
         <v>102</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C57" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
@@ -1267,10 +1275,10 @@
         <v>102</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C58" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
@@ -1278,10 +1286,10 @@
         <v>102</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C59" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
@@ -1289,10 +1297,10 @@
         <v>102</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C60" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
@@ -1300,10 +1308,10 @@
         <v>102</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C61" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
@@ -1311,10 +1319,10 @@
         <v>102</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C62" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
@@ -1322,10 +1330,10 @@
         <v>102</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C63" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
@@ -1333,10 +1341,10 @@
         <v>102</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C64" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
@@ -1344,10 +1352,10 @@
         <v>102</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C65" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
@@ -1355,10 +1363,10 @@
         <v>102</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C66" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
@@ -1366,10 +1374,10 @@
         <v>102</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C67" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
@@ -1377,10 +1385,10 @@
         <v>102</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C68" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
@@ -1388,10 +1396,10 @@
         <v>102</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C69" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
@@ -1399,10 +1407,10 @@
         <v>102</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C70" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
@@ -1410,10 +1418,10 @@
         <v>102</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C71" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
@@ -1421,10 +1429,10 @@
         <v>102</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C72" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
@@ -1432,10 +1440,10 @@
         <v>102</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C73" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
@@ -1443,10 +1451,10 @@
         <v>102</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C74" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
@@ -1454,10 +1462,10 @@
         <v>102</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C75" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
@@ -1465,10 +1473,10 @@
         <v>102</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C76" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
@@ -1476,10 +1484,10 @@
         <v>102</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C77" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
@@ -1487,10 +1495,10 @@
         <v>102</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C78" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
@@ -1498,10 +1506,10 @@
         <v>102</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C79" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
@@ -1509,10 +1517,10 @@
         <v>102</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C80" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
@@ -1520,10 +1528,10 @@
         <v>102</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C81" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
@@ -1531,10 +1539,10 @@
         <v>102</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C82" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
@@ -1542,10 +1550,10 @@
         <v>102</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C83" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
@@ -1553,10 +1561,10 @@
         <v>102</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C84" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
@@ -1564,10 +1572,10 @@
         <v>102</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C85" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
@@ -1575,10 +1583,10 @@
         <v>102</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C86" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
@@ -1586,10 +1594,10 @@
         <v>102</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C87" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
@@ -1597,10 +1605,10 @@
         <v>102</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C88" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
@@ -1608,10 +1616,10 @@
         <v>102</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C89" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
@@ -1619,10 +1627,10 @@
         <v>102</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C90" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
@@ -1630,10 +1638,10 @@
         <v>103</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C91" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
@@ -1641,10 +1649,10 @@
         <v>103</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C92" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
@@ -1652,10 +1660,10 @@
         <v>103</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C93" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
@@ -1663,10 +1671,10 @@
         <v>103</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C94" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
@@ -1674,10 +1682,10 @@
         <v>103</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C95" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
@@ -1685,10 +1693,10 @@
         <v>103</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C96" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
@@ -1696,10 +1704,10 @@
         <v>103</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C97" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
@@ -1707,10 +1715,10 @@
         <v>103</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C98" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
@@ -1718,10 +1726,10 @@
         <v>103</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C99" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
@@ -1729,10 +1737,10 @@
         <v>103</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C100" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
@@ -1740,10 +1748,10 @@
         <v>103</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C101" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
@@ -1751,10 +1759,10 @@
         <v>103</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C102" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
@@ -1762,10 +1770,10 @@
         <v>103</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C103" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
@@ -1773,10 +1781,10 @@
         <v>103</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C104" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
@@ -1784,10 +1792,10 @@
         <v>103</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C105" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
@@ -1795,10 +1803,10 @@
         <v>103</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C106" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
@@ -1806,10 +1814,10 @@
         <v>103</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C107" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
@@ -1817,10 +1825,10 @@
         <v>103</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C108" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
@@ -1828,10 +1836,10 @@
         <v>103</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C109" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
@@ -1839,14 +1847,14 @@
         <v>103</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C110" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>